<commit_message>
260610 update on ppt
</commit_message>
<xml_diff>
--- a/Projects/MISQ/MISQ round 2/writeup/meeting260609_summarization.xlsx
+++ b/Projects/MISQ/MISQ round 2/writeup/meeting260609_summarization.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/dylanchen/Desktop/geek-community/Projects/MISQ/MISQ round 2/writeup/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2712364E-2B8B-4042-939D-43619B734D01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4FA4A1F2-249C-B648-AB98-08566A614B9C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17360" xr2:uid="{30F402B7-E6D8-E34B-8063-713AC97DE139}"/>
   </bookViews>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="918" uniqueCount="391">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="918" uniqueCount="389">
   <si>
     <t>DV: # human answers</t>
   </si>
@@ -1427,28 +1427,22 @@
     <t>Reputation:log_textLengthCN1Ans</t>
   </si>
   <si>
-    <t>-0.120 *</t>
-  </si>
-  <si>
     <t>(0.007)</t>
   </si>
   <si>
-    <t>(0.054)</t>
-  </si>
-  <si>
     <t>-0.013</t>
   </si>
   <si>
     <t>0.350 ***</t>
   </si>
   <si>
-    <t>(0.035)</t>
-  </si>
-  <si>
     <t>first human answer quality (human1SimWithLLMi)</t>
   </si>
   <si>
     <t>2,685</t>
+  </si>
+  <si>
+    <t>-0.120 .</t>
   </si>
 </sst>
 </file>
@@ -3435,10 +3429,10 @@
           <c:layoutTarget val="inner"/>
           <c:xMode val="edge"/>
           <c:yMode val="edge"/>
-          <c:x val="0.12729655775023568"/>
-          <c:y val="4.3437866128041271E-2"/>
-          <c:w val="0.83216836007543871"/>
-          <c:h val="0.82913332350703361"/>
+          <c:x val="0.19658898783623088"/>
+          <c:y val="5.6745720814710666E-2"/>
+          <c:w val="0.75834536036245515"/>
+          <c:h val="0.75926640516999511"/>
         </c:manualLayout>
       </c:layout>
       <c:scatterChart>
@@ -3660,7 +3654,7 @@
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="0.4"/>
-          <c:min val="-0.2"/>
+          <c:min val="-0.1"/>
         </c:scaling>
         <c:delete val="0"/>
         <c:axPos val="l"/>
@@ -3671,7 +3665,7 @@
               <a:lstStyle/>
               <a:p>
                 <a:pPr>
-                  <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:defRPr sz="1800" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
                     <a:solidFill>
                       <a:schemeClr val="tx1">
                         <a:lumMod val="65000"/>
@@ -3684,8 +3678,125 @@
                   </a:defRPr>
                 </a:pPr>
                 <a:r>
-                  <a:rPr lang="en-US"/>
-                  <a:t>7 day #Answer</a:t>
+                  <a:rPr lang="en-US" sz="1800" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0" dirty="0">
+                    <a:solidFill>
+                      <a:prstClr val="black">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:prstClr>
+                    </a:solidFill>
+                  </a:rPr>
+                  <a:t>#</a:t>
+                </a:r>
+                <a:r>
+                  <a:rPr lang="zh-CN" altLang="en-US" sz="1800" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0" dirty="0">
+                    <a:solidFill>
+                      <a:prstClr val="black">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:prstClr>
+                    </a:solidFill>
+                  </a:rPr>
+                  <a:t> </a:t>
+                </a:r>
+                <a:r>
+                  <a:rPr lang="en-US" sz="1800" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0" dirty="0">
+                    <a:solidFill>
+                      <a:prstClr val="black">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:prstClr>
+                    </a:solidFill>
+                  </a:rPr>
+                  <a:t>Human</a:t>
+                </a:r>
+                <a:r>
+                  <a:rPr lang="zh-CN" altLang="en-US" sz="1800" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0" dirty="0">
+                    <a:solidFill>
+                      <a:prstClr val="black">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:prstClr>
+                    </a:solidFill>
+                  </a:rPr>
+                  <a:t> </a:t>
+                </a:r>
+                <a:r>
+                  <a:rPr lang="en-US" sz="1800" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0" dirty="0">
+                    <a:solidFill>
+                      <a:prstClr val="black">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:prstClr>
+                    </a:solidFill>
+                  </a:rPr>
+                  <a:t>Answer</a:t>
+                </a:r>
+                <a:r>
+                  <a:rPr lang="zh-CN" altLang="en-US" sz="1800" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0" dirty="0">
+                    <a:solidFill>
+                      <a:prstClr val="black">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:prstClr>
+                    </a:solidFill>
+                  </a:rPr>
+                  <a:t> </a:t>
+                </a:r>
+                <a:r>
+                  <a:rPr lang="en-US" sz="1800" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0" dirty="0">
+                    <a:solidFill>
+                      <a:prstClr val="black">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:prstClr>
+                    </a:solidFill>
+                  </a:rPr>
+                  <a:t>within</a:t>
+                </a:r>
+                <a:r>
+                  <a:rPr lang="zh-CN" altLang="en-US" sz="1800" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0" dirty="0">
+                    <a:solidFill>
+                      <a:prstClr val="black">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:prstClr>
+                    </a:solidFill>
+                  </a:rPr>
+                  <a:t> </a:t>
+                </a:r>
+                <a:r>
+                  <a:rPr lang="en-US" sz="1800" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0" dirty="0">
+                    <a:solidFill>
+                      <a:prstClr val="black">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:prstClr>
+                    </a:solidFill>
+                  </a:rPr>
+                  <a:t>7</a:t>
+                </a:r>
+                <a:r>
+                  <a:rPr lang="zh-CN" altLang="en-US" sz="1800" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0" dirty="0">
+                    <a:solidFill>
+                      <a:prstClr val="black">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:prstClr>
+                    </a:solidFill>
+                  </a:rPr>
+                  <a:t> </a:t>
+                </a:r>
+                <a:r>
+                  <a:rPr lang="en-US" sz="1800" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0" dirty="0">
+                    <a:solidFill>
+                      <a:prstClr val="black">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:prstClr>
+                    </a:solidFill>
+                  </a:rPr>
+                  <a:t>days</a:t>
                 </a:r>
               </a:p>
             </c:rich>
@@ -3703,7 +3814,7 @@
             <a:lstStyle/>
             <a:p>
               <a:pPr>
-                <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:defRPr sz="1800" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
                   <a:solidFill>
                     <a:schemeClr val="tx1">
                       <a:lumMod val="65000"/>
@@ -3741,7 +3852,7 @@
           <a:lstStyle/>
           <a:p>
             <a:pPr>
-              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:defRPr sz="1800" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
                 <a:solidFill>
                   <a:schemeClr val="tx1">
                     <a:lumMod val="65000"/>
@@ -3766,6 +3877,7 @@
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="7"/>
+          <c:min val="0"/>
         </c:scaling>
         <c:delete val="0"/>
         <c:axPos val="b"/>
@@ -3776,7 +3888,7 @@
               <a:lstStyle/>
               <a:p>
                 <a:pPr>
-                  <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:defRPr sz="1800" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
                     <a:solidFill>
                       <a:schemeClr val="tx1">
                         <a:lumMod val="65000"/>
@@ -3789,19 +3901,19 @@
                   </a:defRPr>
                 </a:pPr>
                 <a:r>
-                  <a:rPr lang="en-US" altLang="zh-CN"/>
+                  <a:rPr lang="en-US"/>
                   <a:t>AI</a:t>
                 </a:r>
                 <a:r>
-                  <a:rPr lang="zh-CN" altLang="en-US"/>
+                  <a:rPr lang="zh-CN"/>
                   <a:t> </a:t>
                 </a:r>
                 <a:r>
-                  <a:rPr lang="en-US" altLang="zh-CN"/>
+                  <a:rPr lang="en-US"/>
                   <a:t>answer</a:t>
                 </a:r>
                 <a:r>
-                  <a:rPr lang="zh-CN" altLang="en-US"/>
+                  <a:rPr lang="zh-CN"/>
                   <a:t> </a:t>
                 </a:r>
                 <a:r>
@@ -3811,6 +3923,14 @@
               </a:p>
             </c:rich>
           </c:tx>
+          <c:layout>
+            <c:manualLayout>
+              <c:xMode val="edge"/>
+              <c:yMode val="edge"/>
+              <c:x val="0.37847856559201215"/>
+              <c:y val="0.90839098154438758"/>
+            </c:manualLayout>
+          </c:layout>
           <c:overlay val="0"/>
           <c:spPr>
             <a:noFill/>
@@ -3824,7 +3944,7 @@
             <a:lstStyle/>
             <a:p>
               <a:pPr>
-                <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:defRPr sz="1800" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
                   <a:solidFill>
                     <a:schemeClr val="tx1">
                       <a:lumMod val="65000"/>
@@ -3862,7 +3982,7 @@
           <a:lstStyle/>
           <a:p>
             <a:pPr>
-              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:defRPr sz="1800" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
                 <a:solidFill>
                   <a:schemeClr val="tx1">
                     <a:lumMod val="65000"/>
@@ -3895,10 +4015,10 @@
         <c:manualLayout>
           <c:xMode val="edge"/>
           <c:yMode val="edge"/>
-          <c:x val="0.74326853131290305"/>
+          <c:x val="0.59825909791468757"/>
           <c:y val="0.10924970324905096"/>
-          <c:w val="0.18846405449128323"/>
-          <c:h val="0.13327620388496833"/>
+          <c:w val="0.3334735333390908"/>
+          <c:h val="0.17773390683414819"/>
         </c:manualLayout>
       </c:layout>
       <c:overlay val="0"/>
@@ -3914,7 +4034,7 @@
         <a:lstStyle/>
         <a:p>
           <a:pPr>
-            <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+            <a:defRPr sz="1800" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
               <a:solidFill>
                 <a:schemeClr val="tx1">
                   <a:lumMod val="65000"/>
@@ -3961,7 +4081,7 @@
     <a:lstStyle/>
     <a:p>
       <a:pPr>
-        <a:defRPr/>
+        <a:defRPr sz="1800"/>
       </a:pPr>
       <a:endParaRPr lang="en-US"/>
     </a:p>
@@ -3995,10 +4115,10 @@
           <c:layoutTarget val="inner"/>
           <c:xMode val="edge"/>
           <c:yMode val="edge"/>
-          <c:x val="0.1511812409357805"/>
+          <c:x val="0.18166413041912891"/>
           <c:y val="4.3874636000693454E-2"/>
-          <c:w val="0.79891442520144573"/>
-          <c:h val="0.8391663253846019"/>
+          <c:w val="0.76843150800609039"/>
+          <c:h val="0.77262652213356342"/>
         </c:manualLayout>
       </c:layout>
       <c:scatterChart>
@@ -4255,7 +4375,7 @@
               <a:lstStyle/>
               <a:p>
                 <a:pPr>
-                  <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:defRPr sz="1800" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
                     <a:solidFill>
                       <a:schemeClr val="tx1">
                         <a:lumMod val="65000"/>
@@ -4268,8 +4388,81 @@
                   </a:defRPr>
                 </a:pPr>
                 <a:r>
-                  <a:rPr lang="en-US"/>
-                  <a:t>Quatlity 1st Human Answer</a:t>
+                  <a:rPr lang="en-US" sz="1800" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0" dirty="0">
+                    <a:solidFill>
+                      <a:prstClr val="black">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:prstClr>
+                    </a:solidFill>
+                  </a:rPr>
+                  <a:t>First</a:t>
+                </a:r>
+                <a:r>
+                  <a:rPr lang="zh-CN" altLang="en-US" sz="1800" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0" dirty="0">
+                    <a:solidFill>
+                      <a:prstClr val="black">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:prstClr>
+                    </a:solidFill>
+                  </a:rPr>
+                  <a:t> </a:t>
+                </a:r>
+                <a:r>
+                  <a:rPr lang="en-US" sz="1800" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0" dirty="0">
+                    <a:solidFill>
+                      <a:prstClr val="black">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:prstClr>
+                    </a:solidFill>
+                  </a:rPr>
+                  <a:t>Human</a:t>
+                </a:r>
+                <a:r>
+                  <a:rPr lang="zh-CN" altLang="en-US" sz="1800" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0" dirty="0">
+                    <a:solidFill>
+                      <a:prstClr val="black">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:prstClr>
+                    </a:solidFill>
+                  </a:rPr>
+                  <a:t> </a:t>
+                </a:r>
+                <a:r>
+                  <a:rPr lang="en-US" sz="1800" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0" dirty="0">
+                    <a:solidFill>
+                      <a:prstClr val="black">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:prstClr>
+                    </a:solidFill>
+                  </a:rPr>
+                  <a:t>Answer</a:t>
+                </a:r>
+                <a:r>
+                  <a:rPr lang="zh-CN" altLang="en-US" sz="1800" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0" dirty="0">
+                    <a:solidFill>
+                      <a:prstClr val="black">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:prstClr>
+                    </a:solidFill>
+                  </a:rPr>
+                  <a:t> </a:t>
+                </a:r>
+                <a:r>
+                  <a:rPr lang="en-US" sz="1800" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0" dirty="0">
+                    <a:solidFill>
+                      <a:prstClr val="black">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:prstClr>
+                    </a:solidFill>
+                  </a:rPr>
+                  <a:t>Quality</a:t>
                 </a:r>
               </a:p>
             </c:rich>
@@ -4287,7 +4480,7 @@
             <a:lstStyle/>
             <a:p>
               <a:pPr>
-                <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:defRPr sz="1800" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
                   <a:solidFill>
                     <a:schemeClr val="tx1">
                       <a:lumMod val="65000"/>
@@ -4325,7 +4518,7 @@
           <a:lstStyle/>
           <a:p>
             <a:pPr>
-              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:defRPr sz="1800" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
                 <a:solidFill>
                   <a:schemeClr val="tx1">
                     <a:lumMod val="65000"/>
@@ -4360,7 +4553,7 @@
               <a:lstStyle/>
               <a:p>
                 <a:pPr>
-                  <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:defRPr sz="1800" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
                     <a:solidFill>
                       <a:schemeClr val="tx1">
                         <a:lumMod val="65000"/>
@@ -4373,19 +4566,19 @@
                   </a:defRPr>
                 </a:pPr>
                 <a:r>
-                  <a:rPr lang="en-US" altLang="zh-CN"/>
+                  <a:rPr lang="en-US"/>
                   <a:t>AI</a:t>
                 </a:r>
                 <a:r>
-                  <a:rPr lang="zh-CN" altLang="en-US"/>
+                  <a:rPr lang="zh-CN"/>
                   <a:t> </a:t>
                 </a:r>
                 <a:r>
-                  <a:rPr lang="en-US" altLang="zh-CN"/>
+                  <a:rPr lang="en-US"/>
                   <a:t>answer</a:t>
                 </a:r>
                 <a:r>
-                  <a:rPr lang="zh-CN" altLang="en-US"/>
+                  <a:rPr lang="zh-CN"/>
                   <a:t> </a:t>
                 </a:r>
                 <a:r>
@@ -4408,7 +4601,7 @@
             <a:lstStyle/>
             <a:p>
               <a:pPr>
-                <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:defRPr sz="1800" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
                   <a:solidFill>
                     <a:schemeClr val="tx1">
                       <a:lumMod val="65000"/>
@@ -4446,7 +4639,7 @@
           <a:lstStyle/>
           <a:p>
             <a:pPr>
-              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:defRPr sz="1800" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
                 <a:solidFill>
                   <a:schemeClr val="tx1">
                     <a:lumMod val="65000"/>
@@ -4479,10 +4672,10 @@
         <c:manualLayout>
           <c:xMode val="edge"/>
           <c:yMode val="edge"/>
-          <c:x val="0.73798715481903754"/>
-          <c:y val="0.67296177301096805"/>
-          <c:w val="0.1898456317965824"/>
-          <c:h val="0.13251545577732426"/>
+          <c:x val="0.59665699735930589"/>
+          <c:y val="0.60974883273512892"/>
+          <c:w val="0.35334525013277662"/>
+          <c:h val="0.16578553657770492"/>
         </c:manualLayout>
       </c:layout>
       <c:overlay val="0"/>
@@ -4498,7 +4691,7 @@
         <a:lstStyle/>
         <a:p>
           <a:pPr>
-            <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+            <a:defRPr sz="1800" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
               <a:solidFill>
                 <a:schemeClr val="tx1">
                   <a:lumMod val="65000"/>
@@ -4545,7 +4738,7 @@
     <a:lstStyle/>
     <a:p>
       <a:pPr>
-        <a:defRPr/>
+        <a:defRPr sz="1800"/>
       </a:pPr>
       <a:endParaRPr lang="en-US"/>
     </a:p>
@@ -13203,8 +13396,8 @@
     <xdr:from>
       <xdr:col>4</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>15</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
+      <xdr:row>13</xdr:row>
+      <xdr:rowOff>50800</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>9</xdr:col>
@@ -13433,8 +13626,8 @@
     <xdr:from>
       <xdr:col>11</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>15</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
+      <xdr:row>13</xdr:row>
+      <xdr:rowOff>50800</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
@@ -15280,7 +15473,7 @@
       </c>
       <c r="D20" s="39"/>
       <c r="E20" s="39" t="s">
-        <v>389</v>
+        <v>386</v>
       </c>
       <c r="F20" s="39"/>
     </row>
@@ -15298,7 +15491,7 @@
         <v>41</v>
       </c>
       <c r="F21" s="13" t="s">
-        <v>383</v>
+        <v>388</v>
       </c>
     </row>
     <row r="22" spans="2:16" x14ac:dyDescent="0.2">
@@ -15310,10 +15503,10 @@
         <v>30</v>
       </c>
       <c r="E22" s="13" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
       <c r="F22" s="13" t="s">
-        <v>385</v>
+        <v>88</v>
       </c>
     </row>
     <row r="23" spans="2:16" ht="16" customHeight="1" x14ac:dyDescent="0.2">
@@ -15326,7 +15519,7 @@
       </c>
       <c r="E23" s="13"/>
       <c r="F23" s="13" t="s">
-        <v>386</v>
+        <v>384</v>
       </c>
     </row>
     <row r="24" spans="2:16" x14ac:dyDescent="0.2">
@@ -15337,7 +15530,7 @@
       </c>
       <c r="E24" s="13"/>
       <c r="F24" s="13" t="s">
-        <v>65</v>
+        <v>16</v>
       </c>
     </row>
     <row r="25" spans="2:16" ht="16" customHeight="1" x14ac:dyDescent="0.2">
@@ -15350,7 +15543,7 @@
       </c>
       <c r="E25" s="13"/>
       <c r="F25" s="13" t="s">
-        <v>387</v>
+        <v>385</v>
       </c>
     </row>
     <row r="26" spans="2:16" x14ac:dyDescent="0.2">
@@ -15361,7 +15554,7 @@
       </c>
       <c r="E26" s="16"/>
       <c r="F26" s="16" t="s">
-        <v>388</v>
+        <v>99</v>
       </c>
     </row>
     <row r="27" spans="2:16" x14ac:dyDescent="0.2">
@@ -15426,10 +15619,10 @@
         <v>347</v>
       </c>
       <c r="E30" s="16" t="s">
-        <v>390</v>
+        <v>387</v>
       </c>
       <c r="F30" s="16" t="s">
-        <v>390</v>
+        <v>387</v>
       </c>
     </row>
     <row r="32" spans="2:16" ht="16" customHeight="1" x14ac:dyDescent="0.2"/>

</xml_diff>